<commit_message>
Add Missing Vulnerability Description for "vuln_sd_failed_sd_read_on_priv-l3" in French
The description is missing on the website. English descriptions taken and translated with Deepl
</commit_message>
<xml_diff>
--- a/tools/excel/anssi/ad/anssi-points-de-controle-active-directory.xlsx
+++ b/tools/excel/anssi/ad/anssi-points-de-controle-active-directory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\tarkadia\projects\intuitem\ciso-assistant-community\tools\excel\anssi\ad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F183799C-DFCA-4D0D-B073-10901FD7A9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E9D49F6-AFB0-4052-965A-378021B370C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30828" yWindow="-4536" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -4284,9 +4284,6 @@
     <t>Comptes privilégiés pour lesquels des informations critiques sont manquantes (Niveau 3)</t>
   </si>
   <si>
-    <t># Description de la vulnérabilité</t>
-  </si>
-  <si>
     <t># Recommandation
 Identifier les raisons pour lesquelles les droits appliqués et les propriétés de ces comptes privilégiés n'ont pu être relevés. Cela peut être dû soit à des droits insuffisants du compte qui a réalisé la collecte ORADAD, soit aux droits positionnés sur les comptes privilégiés ou leurs unités organisationnelles parentes.
 Afin d'effectuer un relevé permettant une analyse exhaustive, il est nécessaire que le compte qui exécute l'outil de relevé (ORADAD) dispose de suffisamment de droits d'accès. En particulier, pour lire le descripteur de sécurité (attribut nTSecurityDescriptor).
@@ -4550,6 +4547,10 @@
   <si>
     <t xml:space="preserve">The Active Directory infrastructure exhibits an enhanced level of security and management;
 </t>
+  </si>
+  <si>
+    <t># Description de la vulnérabilité
+Certaines informations relatives aux comptes privilégiés font défaut. Par conséquent, l'analyse et le niveau de sécurité indiqués dans le présent rapport pourraient être erronés.</t>
   </si>
 </sst>
 </file>
@@ -4585,13 +4586,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4607,6 +4609,26 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7C04E0FD-671E-4DFD-83B0-FB64F3E2A9E0}" name="Tableau1" displayName="Tableau1" ref="A1:K101" totalsRowShown="0">
+  <autoFilter ref="A1:K101" xr:uid="{7C04E0FD-671E-4DFD-83B0-FB64F3E2A9E0}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{E3D446D3-B26F-4A2B-9B48-DF008B6D4C99}" name="assessable"/>
+    <tableColumn id="2" xr3:uid="{4D7F5EBF-E347-4B50-BCE6-9F65C5F7279A}" name="depth"/>
+    <tableColumn id="3" xr3:uid="{2F0069E8-A335-40E7-ADA5-E8781FB5BB6F}" name="node_id"/>
+    <tableColumn id="4" xr3:uid="{468C13FC-0DFE-45A4-A004-B8B454046DA6}" name="ref_id"/>
+    <tableColumn id="5" xr3:uid="{14C27870-0626-4C98-9700-041331142FD2}" name="name"/>
+    <tableColumn id="6" xr3:uid="{7BD25591-3945-4CF4-A82E-8417C6470399}" name="description"/>
+    <tableColumn id="7" xr3:uid="{F402B5F0-7DEF-4FB4-9D0F-5040910FED9D}" name="annotation"/>
+    <tableColumn id="8" xr3:uid="{73042BDA-A2E2-44E5-AA9D-BF5445050DED}" name="implementation_groups"/>
+    <tableColumn id="9" xr3:uid="{A7B6A1DD-0146-4310-8EE5-36F52ECE2747}" name="name[en]"/>
+    <tableColumn id="10" xr3:uid="{C2A9DB7A-2FD0-4F53-B4C5-BA008B74BC85}" name="description[en]"/>
+    <tableColumn id="11" xr3:uid="{AE335DA1-3E24-44E8-9E07-BA3E73A0C586}" name="annotation[en]"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5104,13 +5126,13 @@
   <dimension ref="A1:K101"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" customWidth="1"/>
     <col min="3" max="3" width="28.6640625" customWidth="1"/>
     <col min="4" max="4" width="45.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="109.88671875" customWidth="1"/>
     <col min="6" max="6" width="126.77734375" customWidth="1"/>
     <col min="7" max="7" width="109" customWidth="1"/>
-    <col min="8" max="8" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.21875" customWidth="1"/>
     <col min="9" max="9" width="88.109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="96" customWidth="1"/>
     <col min="11" max="11" width="97.21875" customWidth="1"/>
@@ -8022,7 +8044,7 @@
       <c r="E94" t="s">
         <v>588</v>
       </c>
-      <c r="F94" t="s">
+      <c r="F94" s="4" t="s">
         <v>589</v>
       </c>
       <c r="G94" t="s">
@@ -8054,23 +8076,23 @@
       <c r="E95" t="s">
         <v>595</v>
       </c>
-      <c r="F95" t="s">
+      <c r="F95" s="4" t="s">
+        <v>658</v>
+      </c>
+      <c r="G95" t="s">
         <v>596</v>
-      </c>
-      <c r="G95" t="s">
-        <v>597</v>
       </c>
       <c r="H95" t="s">
         <v>90</v>
       </c>
       <c r="I95" t="s">
+        <v>597</v>
+      </c>
+      <c r="J95" t="s">
         <v>598</v>
       </c>
-      <c r="J95" t="s">
+      <c r="K95" t="s">
         <v>599</v>
-      </c>
-      <c r="K95" t="s">
-        <v>600</v>
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.3">
@@ -8081,28 +8103,28 @@
         <v>38</v>
       </c>
       <c r="D96" t="s">
+        <v>600</v>
+      </c>
+      <c r="E96" t="s">
         <v>601</v>
       </c>
-      <c r="E96" t="s">
+      <c r="F96" t="s">
         <v>602</v>
       </c>
-      <c r="F96" t="s">
+      <c r="G96" t="s">
         <v>603</v>
-      </c>
-      <c r="G96" t="s">
-        <v>604</v>
       </c>
       <c r="H96" t="s">
         <v>90</v>
       </c>
       <c r="I96" t="s">
+        <v>604</v>
+      </c>
+      <c r="J96" t="s">
         <v>605</v>
       </c>
-      <c r="J96" t="s">
+      <c r="K96" t="s">
         <v>606</v>
-      </c>
-      <c r="K96" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.3">
@@ -8113,28 +8135,28 @@
         <v>38</v>
       </c>
       <c r="D97" t="s">
+        <v>607</v>
+      </c>
+      <c r="E97" t="s">
         <v>608</v>
       </c>
-      <c r="E97" t="s">
+      <c r="F97" t="s">
         <v>609</v>
       </c>
-      <c r="F97" t="s">
+      <c r="G97" t="s">
         <v>610</v>
-      </c>
-      <c r="G97" t="s">
-        <v>611</v>
       </c>
       <c r="H97" t="s">
         <v>90</v>
       </c>
       <c r="I97" t="s">
+        <v>611</v>
+      </c>
+      <c r="J97" t="s">
         <v>612</v>
       </c>
-      <c r="J97" t="s">
+      <c r="K97" t="s">
         <v>613</v>
-      </c>
-      <c r="K97" t="s">
-        <v>614</v>
       </c>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.3">
@@ -8145,28 +8167,28 @@
         <v>38</v>
       </c>
       <c r="D98" t="s">
+        <v>614</v>
+      </c>
+      <c r="E98" t="s">
         <v>615</v>
       </c>
-      <c r="E98" t="s">
+      <c r="F98" t="s">
         <v>616</v>
       </c>
-      <c r="F98" t="s">
+      <c r="G98" t="s">
         <v>617</v>
-      </c>
-      <c r="G98" t="s">
-        <v>618</v>
       </c>
       <c r="H98" t="s">
         <v>197</v>
       </c>
       <c r="I98" t="s">
+        <v>618</v>
+      </c>
+      <c r="J98" t="s">
         <v>619</v>
       </c>
-      <c r="J98" t="s">
+      <c r="K98" t="s">
         <v>620</v>
-      </c>
-      <c r="K98" t="s">
-        <v>621</v>
       </c>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.3">
@@ -8177,28 +8199,28 @@
         <v>38</v>
       </c>
       <c r="D99" t="s">
+        <v>621</v>
+      </c>
+      <c r="E99" t="s">
         <v>622</v>
       </c>
-      <c r="E99" t="s">
+      <c r="F99" t="s">
         <v>623</v>
       </c>
-      <c r="F99" t="s">
+      <c r="G99" t="s">
         <v>624</v>
-      </c>
-      <c r="G99" t="s">
-        <v>625</v>
       </c>
       <c r="H99" t="s">
         <v>197</v>
       </c>
       <c r="I99" t="s">
+        <v>625</v>
+      </c>
+      <c r="J99" t="s">
         <v>626</v>
       </c>
-      <c r="J99" t="s">
+      <c r="K99" t="s">
         <v>627</v>
-      </c>
-      <c r="K99" t="s">
-        <v>628</v>
       </c>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.3">
@@ -8209,28 +8231,28 @@
         <v>38</v>
       </c>
       <c r="D100" t="s">
+        <v>628</v>
+      </c>
+      <c r="E100" t="s">
         <v>629</v>
       </c>
-      <c r="E100" t="s">
+      <c r="F100" t="s">
         <v>630</v>
       </c>
-      <c r="F100" t="s">
+      <c r="G100" t="s">
         <v>631</v>
-      </c>
-      <c r="G100" t="s">
-        <v>632</v>
       </c>
       <c r="H100" t="s">
         <v>197</v>
       </c>
       <c r="I100" t="s">
+        <v>632</v>
+      </c>
+      <c r="J100" t="s">
         <v>633</v>
       </c>
-      <c r="J100" t="s">
+      <c r="K100" t="s">
         <v>634</v>
-      </c>
-      <c r="K100" t="s">
-        <v>635</v>
       </c>
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.3">
@@ -8241,32 +8263,35 @@
         <v>38</v>
       </c>
       <c r="D101" t="s">
+        <v>635</v>
+      </c>
+      <c r="E101" t="s">
         <v>636</v>
       </c>
-      <c r="E101" t="s">
+      <c r="F101" t="s">
         <v>637</v>
       </c>
-      <c r="F101" t="s">
+      <c r="G101" t="s">
         <v>638</v>
-      </c>
-      <c r="G101" t="s">
-        <v>639</v>
       </c>
       <c r="H101" t="s">
         <v>197</v>
       </c>
       <c r="I101" t="s">
+        <v>639</v>
+      </c>
+      <c r="J101" t="s">
         <v>640</v>
       </c>
-      <c r="J101" t="s">
+      <c r="K101" t="s">
         <v>641</v>
-      </c>
-      <c r="K101" t="s">
-        <v>642</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -8330,16 +8355,16 @@
         <v>56</v>
       </c>
       <c r="B2" t="s">
+        <v>642</v>
+      </c>
+      <c r="C2" t="s">
         <v>643</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>644</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>645</v>
-      </c>
-      <c r="E2" t="s">
-        <v>646</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -8347,16 +8372,16 @@
         <v>69</v>
       </c>
       <c r="B3" t="s">
+        <v>646</v>
+      </c>
+      <c r="C3" t="s">
         <v>647</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>648</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>649</v>
-      </c>
-      <c r="E3" t="s">
-        <v>650</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -8364,16 +8389,16 @@
         <v>90</v>
       </c>
       <c r="B4" t="s">
+        <v>650</v>
+      </c>
+      <c r="C4" t="s">
         <v>651</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>652</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>653</v>
-      </c>
-      <c r="E4" t="s">
-        <v>654</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -8381,16 +8406,16 @@
         <v>197</v>
       </c>
       <c r="B5" t="s">
+        <v>654</v>
+      </c>
+      <c r="C5" t="s">
         <v>655</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>656</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>657</v>
-      </c>
-      <c r="E5" t="s">
-        <v>658</v>
       </c>
     </row>
   </sheetData>

</xml_diff>